<commit_message>
is yaml valid y fallback
</commit_message>
<xml_diff>
--- a/out/RQ2_architecture_metrics/RQ2_architecture_metrics.xlsx
+++ b/out/RQ2_architecture_metrics/RQ2_architecture_metrics.xlsx
@@ -10,6 +10,8 @@
     <sheet name="response_time" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="input_tokens" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="llm_calls" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="fallback" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="yaml_validity" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -827,4 +829,270 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>arch_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>n_responses</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>n_runs</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>fallback_observed_n</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>fallback_count</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>non_fallback_count</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>fallback_rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>agentic_architecture</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>104</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" t="n">
+        <v>104</v>
+      </c>
+      <c r="E2" t="n">
+        <v>13</v>
+      </c>
+      <c r="F2" t="n">
+        <v>91</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>graph_based_architecture</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>104</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>104</v>
+      </c>
+      <c r="E3" t="n">
+        <v>12</v>
+      </c>
+      <c r="F3" t="n">
+        <v>92</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.1153846153846154</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>one_node_architecture</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>104</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>104</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" t="n">
+        <v>102</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.01923076923076923</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>arch_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>n_responses</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>n_runs</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>yaml_applicable_n</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>yaml_valid_count</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>yaml_invalid_count</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>yaml_missing_n</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>yaml_valid_rate_on_applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>agentic_architecture</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>104</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" t="n">
+        <v>79</v>
+      </c>
+      <c r="E2" t="n">
+        <v>78</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.9873417721518988</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>graph_based_architecture</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>104</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>86</v>
+      </c>
+      <c r="E3" t="n">
+        <v>78</v>
+      </c>
+      <c r="F3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G3" t="n">
+        <v>18</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.9069767441860465</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>one_node_architecture</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>104</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>92</v>
+      </c>
+      <c r="E4" t="n">
+        <v>76</v>
+      </c>
+      <c r="F4" t="n">
+        <v>16</v>
+      </c>
+      <c r="G4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.8260869565217391</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
updated RQ2 fallback metrics
</commit_message>
<xml_diff>
--- a/out/RQ2_architecture_metrics/RQ2_architecture_metrics.xlsx
+++ b/out/RQ2_architecture_metrics/RQ2_architecture_metrics.xlsx
@@ -1034,13 +1034,13 @@
         <v>260</v>
       </c>
       <c r="E2" t="n">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F2" t="n">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1192307692307692</v>
+        <v>0.08846153846153847</v>
       </c>
     </row>
     <row r="3">
@@ -1084,13 +1084,13 @@
         <v>260</v>
       </c>
       <c r="E4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F4" t="n">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="G4" t="n">
-        <v>0.02692307692307692</v>
+        <v>0.01923076923076923</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
a12 implemented in rq2 and rq3_clustering
</commit_message>
<xml_diff>
--- a/out/RQ2_architecture_metrics/RQ2_architecture_metrics.xlsx
+++ b/out/RQ2_architecture_metrics/RQ2_architecture_metrics.xlsx
@@ -12,8 +12,9 @@
     <sheet name="llm_calls" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="code_lines" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="pairwise_wilcoxon" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="fallback" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="yaml_validity" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="pairwise_a12" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="fallback" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="yaml_validity" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1547,7 +1548,7 @@
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>9.839904367816287e-45</v>
+        <v>9.839904367816289e-45</v>
       </c>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="b">
@@ -1787,7 +1788,7 @@
         <v>5506</v>
       </c>
       <c r="P13" t="n">
-        <v>4.604000339103342e-20</v>
+        <v>4.604000339103341e-20</v>
       </c>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="b">
@@ -1805,43 +1806,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>arch_id</t>
+          <t>arch_a</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>n_responses</t>
+          <t>arch_b</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>n_runs</t>
+          <t>metric</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>fallback_observed_n</t>
+          <t>a12_arch_a_over_arch_b</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>fallback_count</t>
+          <t>a12_arch_b_over_arch_a</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>non_fallback_count</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>fallback_rate</t>
+          <t>a12_magnitude</t>
         </is>
       </c>
     </row>
@@ -1851,73 +1847,334 @@
           <t>agentic_architecture</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>255</v>
-      </c>
-      <c r="C2" t="n">
-        <v>5</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>graph_based_architecture</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>answer_code_lines</t>
+        </is>
       </c>
       <c r="D2" t="n">
-        <v>255</v>
+        <v>0.445282583621684</v>
       </c>
       <c r="E2" t="n">
-        <v>17</v>
-      </c>
-      <c r="F2" t="n">
-        <v>238</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.554717416378316</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>negligible</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>graph_based_architecture</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>255</v>
-      </c>
-      <c r="C3" t="n">
-        <v>5</v>
+          <t>agentic_architecture</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>one_node_architecture</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>answer_code_lines</t>
+        </is>
       </c>
       <c r="D3" t="n">
-        <v>255</v>
+        <v>0.4501653210303729</v>
       </c>
       <c r="E3" t="n">
-        <v>9</v>
-      </c>
-      <c r="F3" t="n">
-        <v>246</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.03529411764705882</v>
+        <v>0.5498346789696271</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>negligible</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>graph_based_architecture</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>one_node_architecture</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>255</v>
-      </c>
-      <c r="C4" t="n">
-        <v>5</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>answer_code_lines</t>
+        </is>
       </c>
       <c r="D4" t="n">
-        <v>255</v>
+        <v>0.5116878123798539</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F4" t="n">
-        <v>253</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.007843137254901961</v>
+        <v>0.4883121876201461</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>negligible</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>agentic_architecture</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>graph_based_architecture</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>latency_s</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.7459284890426759</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.2540715109573241</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>agentic_architecture</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>one_node_architecture</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>latency_s</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.8707881584006152</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.1292118415993848</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>graph_based_architecture</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>one_node_architecture</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>latency_s</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.6204998077662438</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.3795001922337562</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>small</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>agentic_architecture</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>graph_based_architecture</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>llm_call_count</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0.8772933487120338</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.1227066512879662</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>agentic_architecture</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>one_node_architecture</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>llm_call_count</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>graph_based_architecture</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>one_node_architecture</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>llm_call_count</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0.9901960784313726</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.009803921568627416</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>agentic_architecture</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>graph_based_architecture</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>total_input_tokens</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0.7771318723567858</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.2228681276432142</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>agentic_architecture</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>one_node_architecture</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>total_input_tokens</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0.5470972702806612</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.4529027297193388</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>negligible</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>graph_based_architecture</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>one_node_architecture</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>total_input_tokens</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0.1845444059976932</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.8154555940023068</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1931,6 +2188,132 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>arch_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>n_responses</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>n_runs</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>fallback_observed_n</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>fallback_count</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>non_fallback_count</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>fallback_rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>agentic_architecture</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>255</v>
+      </c>
+      <c r="C2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" t="n">
+        <v>255</v>
+      </c>
+      <c r="E2" t="n">
+        <v>17</v>
+      </c>
+      <c r="F2" t="n">
+        <v>238</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.06666666666666667</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>graph_based_architecture</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>255</v>
+      </c>
+      <c r="C3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" t="n">
+        <v>255</v>
+      </c>
+      <c r="E3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F3" t="n">
+        <v>246</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.03529411764705882</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>one_node_architecture</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>255</v>
+      </c>
+      <c r="C4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>255</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" t="n">
+        <v>253</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.007843137254901961</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>